<commit_message>
vault backup: 2022-12-21 14:57:46
</commit_message>
<xml_diff>
--- a/Inventar.xlsx
+++ b/Inventar.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_docs\ObsidianNotes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDCE627-31D5-4475-ABE6-2BFEFA991382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357E0DAA-0D47-4A85-A7F0-82011A831754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{92340DE6-C51D-4CE5-B3A8-9BD70AF1859D}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11385" xr2:uid="{92340DE6-C51D-4CE5-B3A8-9BD70AF1859D}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
   <si>
     <t>#</t>
   </si>
@@ -177,6 +177,12 @@
   </si>
   <si>
     <t>sonda P2004MW</t>
+  </si>
+  <si>
+    <t>2000d Kabel</t>
+  </si>
+  <si>
+    <t>Millimess touch proto</t>
   </si>
 </sst>
 </file>
@@ -212,8 +218,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -528,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{040B82F4-9971-4B78-85A0-531FF57D7BB8}">
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -942,7 +949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -953,7 +960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -964,7 +971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -975,7 +982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -986,7 +993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1000,7 +1007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1014,7 +1021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1028,7 +1035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1042,7 +1049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1053,7 +1060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1062,6 +1069,37 @@
       </c>
       <c r="D42">
         <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>47</v>
+      </c>
+      <c r="C43">
+        <v>4346021</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43" s="1">
+        <v>44916</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>48</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+      <c r="E44" s="1">
+        <v>44916</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2022-12-21 15:51:46
</commit_message>
<xml_diff>
--- a/Inventar.xlsx
+++ b/Inventar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_docs\ObsidianNotes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357E0DAA-0D47-4A85-A7F0-82011A831754}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD942D95-8BBE-4849-B18F-666B3277FBF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11385" xr2:uid="{92340DE6-C51D-4CE5-B3A8-9BD70AF1859D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="63">
   <si>
     <t>#</t>
   </si>
@@ -68,27 +68,12 @@
     <t>P-NUCLEO-WB55</t>
   </si>
   <si>
-    <t>pneumat</t>
-  </si>
-  <si>
-    <t>przyg powietrza</t>
-  </si>
-  <si>
-    <t>reg cisn</t>
-  </si>
-  <si>
-    <t>sonda 20</t>
-  </si>
-  <si>
     <t>MarCator 1075R</t>
   </si>
   <si>
     <t>wyslane do sonsalli</t>
   </si>
   <si>
-    <t>N1702VSS</t>
-  </si>
-  <si>
     <t>wyslane do tluczka</t>
   </si>
   <si>
@@ -110,18 +95,12 @@
     <t>DK-D1</t>
   </si>
   <si>
-    <t>DK-D1 stary</t>
-  </si>
-  <si>
     <t>Werksnormal 1283-1 WN</t>
   </si>
   <si>
     <t>NEO3 linux computer</t>
   </si>
   <si>
-    <t>N1702M-HR</t>
-  </si>
-  <si>
     <t>A1701 proto</t>
   </si>
   <si>
@@ -158,18 +137,6 @@
     <t>Millimar N1702M</t>
   </si>
   <si>
-    <t>SSD 512GB Samsung</t>
-  </si>
-  <si>
-    <t>DDRRAM Kingston</t>
-  </si>
-  <si>
-    <t>piersicen 20,024</t>
-  </si>
-  <si>
-    <t>pierscien 20,000</t>
-  </si>
-  <si>
     <t>Sonda P2004U</t>
   </si>
   <si>
@@ -183,6 +150,81 @@
   </si>
   <si>
     <t>Millimess touch proto</t>
+  </si>
+  <si>
+    <t>einstellringe 20,000</t>
+  </si>
+  <si>
+    <t>einstellringe 20,024</t>
+  </si>
+  <si>
+    <t>Düsenmessdorn 20 mit schiebventil</t>
+  </si>
+  <si>
+    <t>N1701 PM 5000:1</t>
+  </si>
+  <si>
+    <t>Wartungseincheit mit Druckminderer 2,0 Bar</t>
+  </si>
+  <si>
+    <t>Schlauch (Düsenmessdorn- N1701)</t>
+  </si>
+  <si>
+    <t>N1701 PF-2500/5000-4</t>
+  </si>
+  <si>
+    <t>Tastatur</t>
+  </si>
+  <si>
+    <t>Rechner Windows 7</t>
+  </si>
+  <si>
+    <t>Rechner Windows 10</t>
+  </si>
+  <si>
+    <t>Bildschirme</t>
+  </si>
+  <si>
+    <t>Maus</t>
+  </si>
+  <si>
+    <t>USB-hub</t>
+  </si>
+  <si>
+    <t>Millimar N1702 VSS</t>
+  </si>
+  <si>
+    <t>Millimar N1702M-HR</t>
+  </si>
+  <si>
+    <t>Retaining Clip board TC2050-CLIP</t>
+  </si>
+  <si>
+    <t>Drehgeber ROD 1080</t>
+  </si>
+  <si>
+    <t>Heidenhein</t>
+  </si>
+  <si>
+    <t>do K. Tluczka</t>
+  </si>
+  <si>
+    <t>Gehäse C1202 mit Glas und Keyboard</t>
+  </si>
+  <si>
+    <t>na wymiane za potluczony</t>
+  </si>
+  <si>
+    <t>Kingston 40KI3232-2016FB</t>
+  </si>
+  <si>
+    <t>Samsung MZ-V8P1T0BW</t>
+  </si>
+  <si>
+    <t>Datenkabel</t>
+  </si>
+  <si>
+    <t>stary kabel 4-pinowy jak DK-D1</t>
   </si>
 </sst>
 </file>
@@ -535,11 +577,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{040B82F4-9971-4B78-85A0-531FF57D7BB8}">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -640,7 +682,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -651,7 +693,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>5331121</v>
@@ -665,7 +707,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C10">
         <v>5331122</v>
@@ -679,7 +721,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>41</v>
+      </c>
+      <c r="C11">
+        <v>5331151</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -690,7 +735,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -701,7 +746,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -712,7 +757,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -723,7 +768,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -734,7 +779,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -745,10 +790,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17">
-        <v>4336010</v>
+        <v>39</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -759,10 +801,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="C18">
-        <v>5312834</v>
+        <v>4336010</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -773,15 +815,12 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>19</v>
+      </c>
+      <c r="C19">
+        <v>5312834</v>
       </c>
       <c r="D19">
-        <v>2</v>
-      </c>
-      <c r="E19" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19">
         <v>1</v>
       </c>
     </row>
@@ -790,13 +829,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D20">
         <v>2</v>
       </c>
       <c r="E20" t="s">
-        <v>17</v>
+        <v>11</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -804,13 +846,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>51</v>
+      </c>
+      <c r="C21">
+        <v>5331161</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -818,10 +863,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D22">
         <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -829,15 +877,9 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23">
         <v>1</v>
       </c>
     </row>
@@ -846,9 +888,15 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24">
         <v>1</v>
       </c>
     </row>
@@ -857,10 +905,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -868,7 +916,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D26">
         <v>2</v>
@@ -879,10 +927,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -890,13 +938,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="C28">
-        <v>9104934</v>
+        <v>4102357</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -904,13 +955,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C29">
-        <v>5323011</v>
+        <v>9104934</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -918,10 +969,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C30">
-        <v>5323013</v>
+        <v>5323011</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -932,7 +983,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>27</v>
+        <v>33</v>
+      </c>
+      <c r="C31">
+        <v>5323013</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -943,7 +997,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -954,7 +1008,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -965,10 +1019,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -976,7 +1030,7 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -987,7 +1041,7 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -998,10 +1052,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>33</v>
-      </c>
-      <c r="C37">
-        <v>4157021</v>
+        <v>25</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -1012,10 +1063,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="C38">
-        <v>4157003</v>
+        <v>4157021</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -1026,10 +1077,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C39">
-        <v>4112713</v>
+        <v>4157003</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -1040,10 +1091,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C40">
-        <v>5331130</v>
+        <v>4112713</v>
       </c>
       <c r="D40">
         <v>1</v>
@@ -1054,7 +1105,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>29</v>
+      </c>
+      <c r="C41">
+        <v>5331130</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -1065,7 +1119,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -1076,16 +1130,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>47</v>
-      </c>
-      <c r="C43">
-        <v>4346021</v>
+        <v>60</v>
       </c>
       <c r="D43">
         <v>1</v>
-      </c>
-      <c r="E43" s="1">
-        <v>44916</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1093,13 +1141,138 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>36</v>
+      </c>
+      <c r="C44">
+        <v>4346021</v>
       </c>
       <c r="D44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" s="1">
         <v>44916</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>37</v>
+      </c>
+      <c r="D45">
+        <v>2</v>
+      </c>
+      <c r="E45" s="1">
+        <v>44916</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>45</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>46</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>47</v>
+      </c>
+      <c r="D48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D49">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>49</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>50</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>53</v>
+      </c>
+      <c r="D52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>54</v>
+      </c>
+      <c r="C53" t="s">
+        <v>55</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="F53" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>57</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="F54" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>